<commit_message>
feat(fe): ask which test-case fields to add
Leave three template columns as ? so candidates can name fields their scenario experience suggests, and ask that question in the cart task description.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/juspeace-fe/public/qa-test/cart-test-case-template.xlsx
+++ b/juspeace-fe/public/qa-test/cart-test-case-template.xlsx
@@ -9,13 +9,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:K30"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="36" customWidth="1"/>
     <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="6" width="36" customWidth="1"/>
     <col min="7" max="8" width="16" customWidth="1"/>
+    <col min="9" max="11" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -59,9 +60,24 @@
           <t>Priority</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H1"/>
+  <autoFilter ref="A1:K1"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" sqref="G2:G30" showErrorMessage="1">
       <formula1>"Pass,Fail,Blocked"</formula1>

</xml_diff>